<commit_message>
enhancement:upgrade , prj model
</commit_message>
<xml_diff>
--- a/worklog/v2.2.2/req/s10/project1.xlsx
+++ b/worklog/v2.2.2/req/s10/project1.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12975"/>
+    <workbookView windowWidth="23040" windowHeight="10695"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -113,7 +113,7 @@
     <t>最后更新时间</t>
   </si>
   <si>
-    <t>最后更新月数</t>
+    <t>最后更新周数</t>
   </si>
   <si>
     <t>填写人</t>

</xml_diff>